<commit_message>
6. MyBenefitsPageTest is in progress.
</commit_message>
<xml_diff>
--- a/Excels/SimpleTherapy_Details.xlsx
+++ b/Excels/SimpleTherapy_Details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Snehal-Vinayak\IdeaProjects\SimpleTherapy_Automation\SimpleTherapy_Web_Automation\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0DBEF3-E97F-4429-B196-5E35827FA825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93A8FF4-2C76-42D5-8DE0-053626955EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{4838E644-DBD1-4BD5-84C0-B33ABF6093BA}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="88">
   <si>
     <t>TitleHeading</t>
   </si>
@@ -216,12 +216,6 @@
     <t>Profile Details</t>
   </si>
   <si>
-    <t>sagar+202601133@mobiuso.com</t>
-  </si>
-  <si>
-    <t>KJTDCYSPMUQVISZKOBHVGQRFOBFCMUDJ</t>
-  </si>
-  <si>
     <t>DOB</t>
   </si>
   <si>
@@ -243,19 +237,70 @@
     <t>FirstName_Updated</t>
   </si>
   <si>
-    <t>Sagar1</t>
-  </si>
-  <si>
     <t>LastName_Updated</t>
   </si>
   <si>
+    <t>Snehal</t>
+  </si>
+  <si>
+    <t>Kadam</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>3' 0"</t>
+  </si>
+  <si>
+    <t>50 lbs</t>
+  </si>
+  <si>
+    <t>Address1_Updated</t>
+  </si>
+  <si>
+    <t>1950 S San Benito St</t>
+  </si>
+  <si>
+    <t>Country_Updated</t>
+  </si>
+  <si>
     <t>City_Updated</t>
   </si>
   <si>
-    <t>Pangale1</t>
-  </si>
-  <si>
-    <t>Fremont1</t>
+    <t>State_Updated</t>
+  </si>
+  <si>
+    <t>Clewiston</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Height_Updated</t>
+  </si>
+  <si>
+    <t>Weight_Updated</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 440 555 5556</t>
+  </si>
+  <si>
+    <t>PhoneNumber_Updated</t>
+  </si>
+  <si>
+    <t>3' 1"</t>
+  </si>
+  <si>
+    <t>51 lbs</t>
+  </si>
+  <si>
+    <t>sagar+202601213@mobiuso.com</t>
+  </si>
+  <si>
+    <t>JJDF4QDPGIXHQVT3JRGUOV3CFJ4FE3D5</t>
   </si>
 </sst>
 </file>
@@ -927,23 +972,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9648E4-D8BC-4082-BED6-0B9F506725CD}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.1796875" style="10" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="10.1796875" style="10" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" style="10" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="9.453125" style="10" customWidth="1" collapsed="1"/>
     <col min="4" max="4" width="28.54296875" style="10" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="5" max="5" width="13.81640625" style="10" customWidth="1"/>
-    <col min="6" max="9" width="10.1796875" style="10" customWidth="1"/>
-    <col min="10" max="10" width="13" style="10" customWidth="1"/>
-    <col min="11" max="11" width="41.08984375" style="10" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="12" max="13" width="17.26953125" style="10" customWidth="1"/>
-    <col min="14" max="14" width="13.26953125" style="10" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="10"/>
+    <col min="5" max="5" width="13.81640625" style="10" customWidth="1" collapsed="1"/>
+    <col min="6" max="9" width="10.1796875" style="10" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="13" style="10" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="40.7265625" style="10" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="13" width="13.26953125" style="10" customWidth="1" collapsed="1"/>
+    <col min="14" max="15" width="17.26953125" style="10" customWidth="1" collapsed="1"/>
+    <col min="16" max="16" width="18.36328125" style="10" customWidth="1" collapsed="1"/>
+    <col min="17" max="17" width="15.26953125" style="10" customWidth="1" collapsed="1"/>
+    <col min="18" max="18" width="12.90625" style="10" customWidth="1" collapsed="1"/>
+    <col min="19" max="19" width="13.08984375" style="10" customWidth="1" collapsed="1"/>
+    <col min="20" max="20" width="20.81640625" style="10" customWidth="1" collapsed="1"/>
+    <col min="21" max="21" width="15.26953125" style="10" customWidth="1" collapsed="1"/>
+    <col min="22" max="22" width="15.1796875" style="10" customWidth="1" collapsed="1"/>
+    <col min="23" max="16384" width="8.7265625" style="10" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>51</v>
       </c>
@@ -960,34 +1012,58 @@
         <v>28</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>29</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>30</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>53</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>52</v>
       </c>
@@ -998,7 +1074,7 @@
         <v>14</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>35</v>
@@ -1007,28 +1083,52 @@
         <v>34700</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>32</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="L2" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>72</v>
+      <c r="P2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>